<commit_message>
feat(x12): add pyx12-backed 850 parser with loop hierarchy and addressing scopes
pyx12 handles tokenization, delimiter detection, and interchange control
checks; the 850 area/loop structure (N1 and PO1 loops) is layered here
since pyx12 ships no 850 map. Loop Context values from the spec resolve
to scopes: qualified loops (N1[ST]), qualified segments (REF[DP]), and
per-occurrence repeating loops (PO1).
</commit_message>
<xml_diff>
--- a/examples/specs/850_reference_spec.xlsx
+++ b/examples/specs/850_reference_spec.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -748,12 +748,27 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>USD</t>
+          <t>CONDITIONAL</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Map the currency only when a buying-party currency code is sent.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CUR01 = 'BY'</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -764,11 +779,6 @@
       <c r="M7" t="inlineStr">
         <is>
           <t>len:3..3</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Defaults to USD when CUR absent.</t>
         </is>
       </c>
     </row>
@@ -1116,17 +1126,32 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CONDITIONAL</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Map the store number only when the ID qualifier is 92 (assigned by buyer).</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>N103 = '92'</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
           <t>string</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Store number (N103 qualifier 92).</t>
         </is>
       </c>
     </row>
@@ -1328,7 +1353,27 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CONDITIONAL</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Map the bill-to ID only when the ID qualifier is 92 (assigned by buyer).</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>N103 = '92'</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -1518,7 +1563,27 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CONDITIONAL</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Map the UPC only when the product ID qualifier is UP.</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>PO106 = 'UP'</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -1529,11 +1594,6 @@
       <c r="M27" t="inlineStr">
         <is>
           <t>len:12..14</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>PO106 qualifier UP.</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1620,27 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CONDITIONAL</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Map the free-form description when the PID is free-form (PID01 = F).</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>PID01 = 'F'</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -1571,11 +1651,6 @@
       <c r="M28" t="inlineStr">
         <is>
           <t>len:1..80</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Item description from the PID inside the PO1 loop.</t>
         </is>
       </c>
     </row>
@@ -1682,6 +1757,85 @@
       <c r="N31" t="inlineStr">
         <is>
           <t>Total transaction amount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>M-031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SAC02</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SAC[A]</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>order.allowance_code</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>len:4..4</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Allowance/charge code (SAC01 = A).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>M-032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>BEG04</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>order.release_number</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Release number; this partner never sends one, default NONE.</t>
         </is>
       </c>
     </row>

</xml_diff>